<commit_message>
Update market journal for 2026-09-09
</commit_message>
<xml_diff>
--- a/Journal_template_2026.xlsx
+++ b/Journal_template_2026.xlsx
@@ -413,7 +413,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -933,7 +933,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1023,7 +1023,7 @@
                 </a:defRPr>
               </a:pPr>
               <a:r>
-                <a:t/>
+                <a:t>None</a:t>
               </a:r>
               <a:endParaRPr lang="en-US"/>
             </a:p>
@@ -1058,7 +1058,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1142,7 +1142,7 @@
                 </a:defRPr>
               </a:pPr>
               <a:r>
-                <a:t/>
+                <a:t>None</a:t>
               </a:r>
               <a:endParaRPr lang="en-US"/>
             </a:p>
@@ -1177,7 +1177,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1215,7 +1215,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -1571,7 +1571,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1633,7 +1633,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1671,7 +1671,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -2000,7 +2000,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2062,7 +2062,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2100,7 +2100,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>

</xml_diff>